<commit_message>
Excepciones en el mapa de trabajo y nombres siempre visibles
- lista_trabajo.xlsx: MOSTRAR (TODO / SOLO LISTA) por departamento y OCULTAR = SI por zona,
  con hoja LEEME. Huancavelica solo muestra lo de la lista.
- Nombres en todos los niveles (también sin elegir nada) y respaldo si falta el centro.
- filtro.js y tooltip.js ya no quedan en caché del navegador.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ZEyFKvQEhXemhLNvQ6ZCJ
</commit_message>
<xml_diff>
--- a/lista_trabajo.xlsx
+++ b/lista_trabajo.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lista" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEEME" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'lista'!$A$1:$D$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'lista'!$A$1:$F$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +31,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,9 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,13 +432,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,6 +464,16 @@
           <t>PROVINCIA</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MOSTRAR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>OCULTAR</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -758,6 +777,11 @@
           <t>HUANCAVELICA</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SOLO LISTA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -885,6 +909,11 @@
           <t>JUNIN</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1459,7 +1488,120 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D47"/>
+  <autoFilter ref="A1:F47"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>CÓMO USAR ESTA LISTA (mapa de trabajo: http://localhost:8000/trabajo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Una fila por zona. Columnas: NOMBRE, NIVEL (DEPARTAMENTO / PROVINCIA / DISTRITO), DEPARTAMENTO, PROVINCIA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Guarda el Excel y recarga la página (F5). No hace falta reiniciar el servidor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MOSTRAR (solo en filas DEPARTAMENTO):</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   TODO        -&gt; se ve el departamento completo (ej. JUNIN).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SOLO LISTA  -&gt; del departamento solo se ven las provincias y distritos que están en esta lista (ej. HUANCAVELICA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OCULTAR = SI (en cualquier fila PROVINCIA o DISTRITO):</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   esa zona no se dibuja en el mapa (excepción), aunque su departamento esté en TODO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ejemplos:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Agregar un distrito:   LIRCAY | DISTRITO | HUANCAVELICA | ANGARAES</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Quitar un distrito:    'TAPO | DISTRITO | JUNIN | TARMA | | SI'   (o borra su fila)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Quitar una provincia de Junín:  'SATIPO | PROVINCIA | JUNIN | SATIPO | | SI'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Si una fila sale con ⚠ 'no encontrado' en el panel, revisa cómo está escrito el nombre (las tildes y la Ñ no importan).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Burbujas de sedes dentro de su distrito y Chanchamayo/Satipo ocultos
- DimDependencia trae coordenadas con errores de tipeo (Chupaca -7517.975, Concepción
  -14.926...): solo se usan las que caen dentro del distrito (mediana); si no, el centro
  del distrito. Las descartadas salen en los avisos del panel.
- lista_trabajo.xlsx: OCULTAR = SI en Chanchamayo y Satipo (sin jueces en la hoja Provincias).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ZEyFKvQEhXemhLNvQ6ZCJ
</commit_message>
<xml_diff>
--- a/lista_trabajo.xlsx
+++ b/lista_trabajo.xlsx
@@ -540,6 +540,11 @@
           <t>CHANCHAMAYO</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1330,6 +1335,11 @@
       <c r="D40" t="inlineStr">
         <is>
           <t>SATIPO</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1522,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1527,7 +1536,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1549,7 +1557,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1564,7 +1571,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -1593,7 +1599,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>

</xml_diff>